<commit_message>
average nearest-island distance, updated plots w/ new features
</commit_message>
<xml_diff>
--- a/Example_data/OUTPUT-1channel_frozen/data_leaf_damage_singlemetrics.xlsx
+++ b/Example_data/OUTPUT-1channel_frozen/data_leaf_damage_singlemetrics.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,55 +449,60 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>total_interisland_distances</t>
+          <t>total_nearest_island_distances</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>mean_nearest_island_distance</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>island_counts</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>total_leaf_size_px</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>total_leaf_size_cm2</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>total_damage_area_px</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>total_damage_area_cm2</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>total_damage_percentage</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>threshold_val_leaf</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>threshold_val_dmg</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>background_leaf</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>background_dmg</t>
         </is>
@@ -532,33 +537,36 @@
         <v>199.2340063194676</v>
       </c>
       <c r="H2" t="n">
+        <v>7.6628463969026</v>
+      </c>
+      <c r="I2" t="n">
         <v>26</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>26847</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>1.564419322883282</v>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>4731</v>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>0.2756832352427015</v>
       </c>
-      <c r="M2" t="n">
+      <c r="N2" t="n">
         <v>17.62208067940552</v>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>5</v>
       </c>
-      <c r="O2" t="n">
+      <c r="P2" t="n">
         <v>78</v>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>2</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>39</v>
       </c>
     </row>
@@ -591,33 +599,36 @@
         <v>163.2220354262268</v>
       </c>
       <c r="H3" t="n">
+        <v>10.88146902841512</v>
+      </c>
+      <c r="I3" t="n">
         <v>15</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>23287</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>1.356972204416992</v>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>3728</v>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>0.217236757764699</v>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>16.00893202215829</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>6</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>134</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>2</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>67</v>
       </c>
     </row>
@@ -650,33 +661,36 @@
         <v>139.5221817229474</v>
       </c>
       <c r="H4" t="n">
+        <v>7.34327272226039</v>
+      </c>
+      <c r="I4" t="n">
         <v>19</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>25388</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>1.479400967309597</v>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>7819</v>
       </c>
-      <c r="L4" t="n">
+      <c r="M4" t="n">
         <v>0.4556261290134608</v>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>30.79801481014652</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>5</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>84</v>
       </c>
-      <c r="P4" t="n">
-        <v>1</v>
-      </c>
       <c r="Q4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R4" t="n">
         <v>42</v>
       </c>
     </row>
@@ -709,33 +723,36 @@
         <v>126.431509133984</v>
       </c>
       <c r="H5" t="n">
+        <v>7.901969320873998</v>
+      </c>
+      <c r="I5" t="n">
         <v>16</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>25501</v>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>1.485985665171027</v>
       </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
         <v>7904</v>
       </c>
-      <c r="L5" t="n">
+      <c r="M5" t="n">
         <v>0.4605792203251559</v>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>30.99486294655112</v>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>6</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>88</v>
       </c>
-      <c r="P5" t="n">
-        <v>1</v>
-      </c>
       <c r="Q5" t="n">
+        <v>1</v>
+      </c>
+      <c r="R5" t="n">
         <v>44</v>
       </c>
     </row>

</xml_diff>